<commit_message>
Refresh match exports — 199/207 completed, 8 U-18 matches remaining
https://claude.ai/code/session_0148r3z4qev5CHYD3aeZjDqW
</commit_message>
<xml_diff>
--- a/west_zone_pickleball_2026_results.xlsx
+++ b/west_zone_pickleball_2026_results.xlsx
@@ -760,10 +760,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
@@ -786,7 +786,7 @@
         <v>23</v>
       </c>
       <c r="E16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2571,7 +2571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3171,11 +3171,19 @@
           <t>Kartik Modi</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>11-2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Piyush Gaikwad</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -3196,11 +3204,19 @@
           <t>Ansh Goyal</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>11-10</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Harikesh Sanghai</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -3287,11 +3303,19 @@
           <t>Kartik Modi</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>11-3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Harikesh Sanghai</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -3312,11 +3336,19 @@
           <t>Jay Agrawal</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>4-11</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Jay Agrawal</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3692,7 +3724,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Piyush Gaikwad</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3700,11 +3732,19 @@
           <t>Sahaj Agrawal</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>11-2</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Piyush Gaikwad</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -3717,7 +3757,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Jay Agrawal</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3729,7 +3769,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -3780,14 +3820,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+          <t>Piyush Gaikwad</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>7-11</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Piyush Gaikwad</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -3816,6 +3864,31 @@
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Finals</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Piyush Gaikwad</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4630,11 +4703,19 @@
           <t>Kavya Nandardhane</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>17-15</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Anjali</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -4650,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4722,11 +4803,19 @@
           <t>Jinisha &amp; Shryesh</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Jinisha &amp; Shryesh</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -4747,11 +4836,19 @@
           <t>Kashish &amp; Aaksh</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>11-10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sasha Salvi &amp; Dhanush Thakur</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -4772,11 +4869,19 @@
           <t>Jinisha &amp; Shryesh</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>4-11</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Jinisha &amp; Shryesh</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -4797,11 +4902,19 @@
           <t>Laxmi Zambre &amp; Atharv Dandage</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4-11</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Laxmi Zambre &amp; Atharv Dandage</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -4814,19 +4927,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Aarav &amp; Sarrah</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Anjali &amp; Jay Agrawal</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Riddhima Gungewad &amp; Bhuvan Gewad</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>6-11</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Anjali &amp; Jay Agrawal</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -4844,17 +4965,158 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>Riddhima Gungewad &amp; Bhuvan Gewad</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>11-7</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Anjali &amp; Jay Agrawal</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Aarav &amp; Sarrah</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Laxmi Zambre &amp; Atharv Dandage</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>11-1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Aarav &amp; Sarrah</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Anjali &amp; Jay Agrawal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Laxmi Zambre &amp; Atharv Dandage</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Aarav &amp; Sarrah</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Riddhima Gungewad &amp; Bhuvan Gewad</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jinisha &amp; Shryesh</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Sasha Salvi &amp; Dhanush Thakur</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh all-3-day match data (14 categories, 204/207 completed)
Confirmed the tournament has 14 categories total across all three days
(29-31 May); dateTab is a UI filter only and each category payload already
contains its full match list, so this is the complete multi-day dataset.

https://claude.ai/code/session_0148r3z4qev5CHYD3aeZjDqW
</commit_message>
<xml_diff>
--- a/west_zone_pickleball_2026_results.xlsx
+++ b/west_zone_pickleball_2026_results.xlsx
@@ -763,7 +763,7 @@
         <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16">
@@ -809,7 +809,7 @@
         <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3765,11 +3765,19 @@
           <t>Aarav Mandal</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>11-3</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Jay Agrawal</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -3848,7 +3856,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Jay Agrawal</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3856,11 +3864,19 @@
           <t>Shreyas Rajaram</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>11-8</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Jay Agrawal</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -3878,14 +3894,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Jay Agrawal</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -5034,11 +5050,19 @@
           <t>Laxmi Zambre &amp; Atharv Dandage</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>11-6</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Anjali &amp; Jay Agrawal</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -5059,11 +5083,19 @@
           <t>Riddhima Gungewad &amp; Bhuvan Gewad</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>11-2</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Aarav &amp; Sarrah</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -5081,14 +5113,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Aarav &amp; Sarrah</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -5101,7 +5133,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Anjali &amp; Jay Agrawal</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5113,7 +5145,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>

</xml_diff>

<commit_message>
Add missing U-12 Girls Doubles category; refresh full dataset
The tournament (link /233df) is a single record with 15 youth categories
spanning 29-31 May. Each category payload already contains its complete
match list across all days, so the day tabs are a UI filter only. Added the
previously-missing U-12 Girls Doubles (not linked on the landing page but a
valid category). Now 15 categories, 210 matches, 207 completed, 3 finals left.

https://claude.ai/code/session_0148r3z4qev5CHYD3aeZjDqW
</commit_message>
<xml_diff>
--- a/west_zone_pickleball_2026_results.xlsx
+++ b/west_zone_pickleball_2026_results.xlsx
@@ -11,17 +11,18 @@
     <sheet name="U-12 Boys Doubles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="U-12 Girls Singles" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="U-12 Mixed Doubles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="U-12 Boys Singles" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="U-14 Girls Doubles" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="U-14 Boys Doubles" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="U-14 Boys Singles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="U-14 Girls Singles" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="U-14 Mixed Doubles" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="U-18 Boys Doubles" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="U-18 Girls Doubles" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="U-18 Boys Singles" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="U-18 Girls Singles" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="U-18 Mixed Doubles" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="U-12 Girls Doubles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="U-12 Boys Singles" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="U-14 Girls Doubles" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="U-14 Boys Doubles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="U-14 Boys Singles" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="U-14 Girls Singles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="U-14 Mixed Doubles" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="U-18 Boys Doubles" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="U-18 Girls Doubles" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="U-18 Boys Singles" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="U-18 Girls Singles" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="U-18 Mixed Doubles" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -562,30 +563,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U-12 Boys Singles</t>
+          <t>U-12 Girls Doubles</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11 AM</t>
+          <t>9 AM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>roundRobinKnockout</t>
+          <t>roundRobin</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>U-14 Girls Doubles</t>
+          <t>U-12 Boys Singles</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -599,62 +600,62 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U-14 Boys Doubles</t>
+          <t>U-14 Girls Doubles</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12 PM</t>
+          <t>11 AM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>roundRobin</t>
+          <t>roundRobinKnockout</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>U-14 Boys Singles</t>
+          <t>U-14 Boys Doubles</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1 PM</t>
+          <t>12 PM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>roundRobinKnockout</t>
+          <t>roundRobin</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>U-14 Girls Singles</t>
+          <t>U-14 Boys Singles</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -668,21 +669,21 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>U-14 Mixed Doubles</t>
+          <t>U-14 Girls Singles</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2:30 PM</t>
+          <t>1 PM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -691,21 +692,21 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E12" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>U-18 Boys Doubles</t>
+          <t>U-14 Mixed Doubles</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3 PM</t>
+          <t>2:30 PM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -714,16 +715,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>U-18 Girls Doubles</t>
+          <t>U-18 Boys Doubles</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -737,21 +738,21 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>U-18 Boys Singles</t>
+          <t>U-18 Girls Doubles</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>5 PM</t>
+          <t>3 PM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -760,16 +761,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E15" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U-18 Girls Singles</t>
+          <t>U-18 Boys Singles</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -783,32 +784,55 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="E16" t="n">
-        <v>23</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>U-18 Girls Singles</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>5 PM</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>roundRobinKnockout</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>23</v>
+      </c>
+      <c r="E17" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>U-18 Mixed Doubles</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>7 PM</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>roundRobinKnockout</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>11</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>9</v>
       </c>
     </row>
@@ -818,6 +842,708 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>U-14 Girls Singles  |  1 PM  |  roundRobinKnockout  |  29 May 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Team 1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Team 2</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool A)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Varun Chopra</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Walkover</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool A)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Varun Chopra</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>11-0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Walkover</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool A)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kanak</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>11-9</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Kanak</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tvisha Shah</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool B)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tvisha Shah</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Kanak</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>8-11</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Kanak</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool C)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Arohi Jagdale</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rashida Lokhandwala</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>12-10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Arohi Jagdale</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool C)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rashida Lokhandwala</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>11-9</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool C)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Arohi Jagdale</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Arohi Jagdale</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool D)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Aadya Vinod</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kimayaa Bholane</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>11-8</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Aadya Vinod</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool D)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mitali Amol Ghodke</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kimayaa Bholane</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kimayaa Bholane</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Round Robin (Pool D)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mitali Amol Ghodke</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Aadya Vinod</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Aadya Vinod</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kimayaa Bholane</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>11-0</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kanak</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>11-8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Arohi Jagdale</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Aadya Vinod</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>11-9</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Demeera Gupta</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>11-0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Kalash</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>6-11</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Finals</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>12-15</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Aaradhya Satpute</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1643,7 +2369,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2205,7 +2931,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2565,7 +3291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3911,7 +4637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4741,7 +5467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5758,6 +6484,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>U-12 Girls Doubles  |  9 AM  |  roundRobin  |  29 May 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Team 1</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Team 2</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>(no match data available yet)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6314,7 +7114,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6678,7 +7478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7075,7 +7875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7866,706 +8666,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>U-14 Girls Singles  |  1 PM  |  roundRobinKnockout  |  29 May 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Team 1</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Team 2</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Winner</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool A)</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Varun Chopra</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0-11</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Walkover</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool A)</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Varun Chopra</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>11-0</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Walkover</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool A)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>8-11</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool B)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Kanak</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>11-9</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Kanak</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool B)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tvisha Shah</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>0-11</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool B)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Tvisha Shah</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Kanak</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>8-11</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Kanak</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool C)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Arohi Jagdale</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Rashida Lokhandwala</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>12-10</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Arohi Jagdale</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool C)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Rashida Lokhandwala</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>11-9</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool C)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Arohi Jagdale</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>1-11</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Arohi Jagdale</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool D)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Aadya Vinod</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Kimayaa Bholane</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>11-8</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Aadya Vinod</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool D)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Mitali Amol Ghodke</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Kimayaa Bholane</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>3-11</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Kimayaa Bholane</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Round Robin (Pool D)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Mitali Amol Ghodke</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Aadya Vinod</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2-11</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Aadya Vinod</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Quarter Finals</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Kimayaa Bholane</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>11-0</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Quarter Finals</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Kanak</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>11-8</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Quarter Finals</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Arohi Jagdale</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>10-11</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Quarter Finals</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Aadya Vinod</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>11-9</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Semi Finals</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Demeera Gupta</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>11-0</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Semi Finals</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Kalash</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>6-11</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Finals</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Sanchi Khillare</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>12-15</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Aaradhya Satpute</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add completed-only export (410 finished matches across 3 days)
New west_zone_pickleball_2026_COMPLETED.xlsx contains only COMPLETED matches:
a Summary tab, a flat 'All Completed' sheet (410 rows), and one tab per
category. Also adds match_results_csv/ALL_completed_matches.csv.

https://claude.ai/code/session_0148r3z4qev5CHYD3aeZjDqW
</commit_message>
<xml_diff>
--- a/west_zone_pickleball_2026_results.xlsx
+++ b/west_zone_pickleball_2026_results.xlsx
@@ -869,13 +869,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D21" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -911,13 +911,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -935,10 +935,10 @@
         <v>45</v>
       </c>
       <c r="D24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -974,13 +974,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -5337,7 +5337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5673,11 +5673,19 @@
           <t>Aniket Durgawali &amp; Bhumika</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>11-4</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ajay Chaudhari &amp; Anuja Maheshwari</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -5794,14 +5802,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+          <t>Aniket Durgawali &amp; Bhumika</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>15-5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Vanshik Kapadia &amp; Vrushali Thakare</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -5814,7 +5830,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Ajay Chaudhari &amp; Anuja Maheshwari</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5822,14 +5838,55 @@
           <t>Shreyas Rajaram &amp; Arpana Choudhary</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>15-7</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ajay Chaudhari &amp; Anuja Maheshwari</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Finals</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Vanshik Kapadia &amp; Vrushali Thakare</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ajay Chaudhari &amp; Anuja Maheshwari</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>15-7</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Vanshik Kapadia &amp; Vrushali Thakare</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7997,7 +8054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8168,11 +8225,19 @@
           <t>Ananda Mandala &amp; Nidhi Saxena</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ananda Mandala &amp; Nidhi Saxena</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -8193,11 +8258,19 @@
           <t>Ananda Mandala &amp; Nidhi Saxena</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ananda Mandala &amp; Nidhi Saxena</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -8248,14 +8321,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+          <t>Akshay Sachdev &amp; Sujata Gupta</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>11-10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Babita Saini &amp; Srijith Shivan</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -8268,7 +8349,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Ananda Mandala &amp; Nidhi Saxena</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -8276,14 +8357,55 @@
           <t>Gayatri Mewada &amp; Chakradhar</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>11-4</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ananda Mandala &amp; Nidhi Saxena</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Finals</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Babita Saini &amp; Srijith Shivan</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ananda Mandala &amp; Nidhi Saxena</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>15-9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Babita Saini &amp; Srijith Shivan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9832,11 +9954,19 @@
           <t>Nikhil Soni &amp; Vaibhav Wavade</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>15-4</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Aarav Mandal &amp; Aadit Palresha</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -10216,7 +10346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10519,11 +10649,19 @@
           <t>Sashikant Singh &amp; Manasi Narade</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>11-4</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Anshika Kanojia &amp; Yash Sharma</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -11072,11 +11210,19 @@
           <t>Navya Bhise &amp; Navya Bhise</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>11-5</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Aarav Mandal &amp; Sarrah Hakim</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -11122,7 +11268,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Anshika Kanojia &amp; Yash Sharma</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -11130,11 +11276,19 @@
           <t>Srijith Shivan &amp; Babita Saini</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>5-11</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -11155,11 +11309,19 @@
           <t>Richa Bhansali &amp; Rajat Parmar</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>11-2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Aishwarya &amp; Bhushan Baviskar</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -11180,11 +11342,19 @@
           <t>Hozaifa Hakim &amp; Asha Eapen</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>11-2</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Shauri Jain &amp; Akshay Sachdev</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -11202,14 +11372,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+          <t>Sashikant Singh &amp; Manasi Narade</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>11-5</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare &amp; Laksh Khillare</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -11230,11 +11408,19 @@
           <t>Sakhi Sinha &amp; Yashovardhan Jibhkate</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>11-1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Shishir Lanke &amp; Rashmi Kulkarni</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -11255,11 +11441,19 @@
           <t>Suchisattam Saran &amp; Aparna Amnerkar</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>11-10</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -11272,7 +11466,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Aarav Mandal &amp; Sarrah Hakim</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -11280,14 +11474,220 @@
           <t>Dhanush Thakur &amp; Sasha Salvi</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>11-9</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Aarav Mandal &amp; Sarrah Hakim</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Aishwarya &amp; Bhushan Baviskar</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>11-4</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Shauri Jain &amp; Akshay Sachdev</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sanchi Khillare &amp; Laksh Khillare</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>11-5</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Shauri Jain &amp; Akshay Sachdev</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Quarter Finals</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Shishir Lanke &amp; Rashmi Kulkarni</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>9-11</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Aarav Mandal &amp; Sarrah Hakim</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Semi Finals</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Shauri Jain &amp; Akshay Sachdev</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>10-11</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Finals</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Mahima Bharsawde &amp; Ramit Desai</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>11-4</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Srijith Shivan &amp; Babita Saini</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>